<commit_message>
A11: Receivables Aging report (AccGenie)
New "Receivables Aging" report — how old each debtor's outstanding is.
AccGenie is balance-based (no open-item tracking), so aging uses FIFO:
a debtor's total receipts are applied against its charges oldest-
first; the unpaid remainder of each charge is bucketed 0-30 / 31-60 /
61-90 / 90+ days from the report date. A Dr opening balance is the
oldest charge.

- core/reports_engine.py — receivables_aging(as_of); verified with a
  FIFO smoke test.
- ui/reports_page.py — ReceivablesAgingPage (as-of report, per-debtor
  buckets + TOTAL row).
- core/exporters.py — Excel + PDF receivables_aging exporters.
- main_window — registered in report_specs (gated, STANDARD-tier).
- make_config_xlsx.py — receivables_aging feature flag under Reports
  (auto STANDARD/PRO/PREMIUM via ALL_REPORT_FEATURES); regenerated
  pricing.xlsx + rebaked.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/pricing.xlsx
+++ b/config/pricing.xlsx
@@ -700,7 +700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H38"/>
+  <dimension ref="A1:H39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1336,12 +1336,12 @@
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>Output</t>
+          <t>Reports</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>export_excel</t>
+          <t>receivables_aging</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
@@ -1379,7 +1379,7 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>export_pdf</t>
+          <t>export_excel</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
@@ -1417,7 +1417,7 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>print</t>
+          <t>export_pdf</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
@@ -1455,7 +1455,7 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>email_report</t>
+          <t>print</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
@@ -1488,12 +1488,12 @@
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>Reconciliation</t>
+          <t>Output</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>bank_reconciliation</t>
+          <t>email_report</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>bank_reco_split</t>
+          <t>bank_reconciliation</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
@@ -1569,7 +1569,7 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>ledger_reconciliation</t>
+          <t>bank_reco_split</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
@@ -1607,7 +1607,7 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>ledger_reco_split</t>
+          <t>ledger_reconciliation</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
@@ -1640,12 +1640,12 @@
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>Migration</t>
+          <t>Reconciliation</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>book_migration</t>
+          <t>ledger_reco_split</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
@@ -1678,12 +1678,12 @@
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>Tax</t>
+          <t>Migration</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>gst</t>
+          <t>book_migration</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
@@ -1692,7 +1692,11 @@
         </is>
       </c>
       <c r="D30" s="5" t="n"/>
-      <c r="E30" s="5" t="n"/>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
           <t>Y</t>
@@ -1705,7 +1709,7 @@
       </c>
       <c r="H30" s="5" t="inlineStr">
         <is>
-          <t>PRO</t>
+          <t>STANDARD</t>
         </is>
       </c>
     </row>
@@ -1717,7 +1721,7 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>tds</t>
+          <t>gst</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
@@ -1746,12 +1750,12 @@
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Tax</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>ai_document_reader</t>
+          <t>tds</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
@@ -1785,7 +1789,7 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>verbal_entry</t>
+          <t>ai_document_reader</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
@@ -1819,7 +1823,7 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>auto_billing</t>
+          <t>verbal_entry</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
@@ -1848,12 +1852,12 @@
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>Enterprise</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>whatsapp</t>
+          <t>auto_billing</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
@@ -1863,7 +1867,11 @@
       </c>
       <c r="D35" s="5" t="n"/>
       <c r="E35" s="5" t="n"/>
-      <c r="F35" s="5" t="n"/>
+      <c r="F35" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
           <t>Y</t>
@@ -1871,7 +1879,7 @@
       </c>
       <c r="H35" s="5" t="inlineStr">
         <is>
-          <t>PREMIUM</t>
+          <t>PRO</t>
         </is>
       </c>
     </row>
@@ -1883,7 +1891,7 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>audit_export</t>
+          <t>whatsapp</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
@@ -1913,7 +1921,7 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>api_access</t>
+          <t>audit_export</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
@@ -1943,7 +1951,7 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>verticals</t>
+          <t>api_access</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
@@ -1960,6 +1968,36 @@
         </is>
       </c>
       <c r="H38" s="5" t="inlineStr">
+        <is>
+          <t>PREMIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>Enterprise</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>verticals</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="n"/>
+      <c r="E39" s="5" t="n"/>
+      <c r="F39" s="5" t="n"/>
+      <c r="G39" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H39" s="5" t="inlineStr">
         <is>
           <t>PREMIUM</t>
         </is>
@@ -1971,10 +2009,10 @@
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="C5:G38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C5:G39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Y,"</formula1>
     </dataValidation>
-    <dataValidation sqref="H5:H38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"DEMO,FREE,STANDARD,PRO,PREMIUM"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Pricing: add bill_wise_refs (PRO+), payables_aging (STD+), cash_flow_planning (PRO+)
New paid-feature flags added to config/pricing.xlsx PlanFeatures and baked
into core/ + license_server/ _baked_config:
- bill_wise_refs       -> PRO, PREMIUM   (Tally "Against Reference" billing)
- payables_aging       -> STANDARD+      (sibling of receivables_aging)
- cash_flow_planning   -> PRO, PREMIUM   (aging -> projected cash / funds gap)

Flags only — the features themselves are TODO (tracked in memory). Gating
verified: FREE excluded; STANDARD has payables_aging only; PRO/PREMIUM have
all three.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/pricing.xlsx
+++ b/config/pricing.xlsx
@@ -740,7 +740,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:H44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="14" customWidth="1" style="10" min="1" max="1"/>
@@ -2122,6 +2122,107 @@
         </is>
       </c>
       <c r="H41" t="inlineStr">
+        <is>
+          <t>PRO</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Accounting</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>bill_wise_refs</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>PRO</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Reports</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>payables_aging</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Reports</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>cash_flow_planning</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
         <is>
           <t>PRO</t>
         </is>

</xml_diff>